<commit_message>
all edited for sir and bhotange merged
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/thekka/घुम्ती खनाल टोल सडक/घुम्ती खनाल टोल सडक.xlsx
+++ b/बजेट माग estimate/thekka/घुम्ती खनाल टोल सडक/घुम्ती खनाल टोल सडक.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B50F655-0E9D-4C1D-9B2F-78CE412BD5D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20736" windowHeight="11040"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="estimate" sheetId="14" r:id="rId1"/>
@@ -39,7 +40,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">estimate!$A$1:$K$75</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">estimate!$1:$8</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -258,10 +259,10 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="14" x14ac:knownFonts="1">
     <font>
@@ -421,9 +422,9 @@
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
@@ -435,7 +436,7 @@
     <xf numFmtId="1" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -459,14 +460,14 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="43" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -485,7 +486,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -500,7 +501,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -516,25 +517,10 @@
     <xf numFmtId="0" fontId="12" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -555,17 +541,32 @@
     <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Comma 2" xfId="3"/>
+    <cellStyle name="Comma 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="2"/>
-    <cellStyle name="Normal 3" xfId="5"/>
-    <cellStyle name="Percent 2" xfId="4"/>
+    <cellStyle name="Normal 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
+    <cellStyle name="Normal 3" xfId="5" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
+    <cellStyle name="Percent 2" xfId="4" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
@@ -581,7 +582,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -675,7 +676,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -734,7 +735,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -798,9 +799,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -838,9 +839,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -875,7 +876,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -910,7 +911,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1083,135 +1084,135 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:S75"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.6640625" style="19" customWidth="1"/>
-    <col min="2" max="2" width="30.88671875" style="19" customWidth="1"/>
-    <col min="3" max="3" width="4.44140625" style="19" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.44140625" style="19" customWidth="1"/>
-    <col min="5" max="5" width="8.5546875" style="19" customWidth="1"/>
-    <col min="6" max="6" width="7.33203125" style="19" customWidth="1"/>
-    <col min="7" max="7" width="9.109375" style="19"/>
+    <col min="1" max="1" width="4.7109375" style="19" customWidth="1"/>
+    <col min="2" max="2" width="30.85546875" style="19" customWidth="1"/>
+    <col min="3" max="3" width="4.42578125" style="19" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.42578125" style="19" customWidth="1"/>
+    <col min="5" max="5" width="8.5703125" style="19" customWidth="1"/>
+    <col min="6" max="6" width="7.28515625" style="19" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" style="19"/>
     <col min="8" max="8" width="5" style="19" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.5546875" style="19" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.6640625" style="19" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="9.109375" style="19"/>
+    <col min="9" max="9" width="9.5703125" style="19" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="9.140625" style="19"/>
     <col min="13" max="16" width="0" style="19" hidden="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.109375" style="19"/>
+    <col min="17" max="16384" width="9.140625" style="19"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A1" s="40" t="s">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
-      <c r="I1" s="40"/>
-      <c r="J1" s="40"/>
-      <c r="K1" s="40"/>
-    </row>
-    <row r="2" spans="1:16" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="41" t="s">
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="48"/>
+    </row>
+    <row r="2" spans="1:16" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="41"/>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41"/>
-      <c r="I2" s="41"/>
-      <c r="J2" s="41"/>
-      <c r="K2" s="41"/>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A3" s="42" t="s">
+      <c r="B2" s="49"/>
+      <c r="C2" s="49"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="49"/>
+      <c r="F2" s="49"/>
+      <c r="G2" s="49"/>
+      <c r="H2" s="49"/>
+      <c r="I2" s="49"/>
+      <c r="J2" s="49"/>
+      <c r="K2" s="49"/>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A3" s="50" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="42"/>
-      <c r="C3" s="42"/>
-      <c r="D3" s="42"/>
-      <c r="E3" s="42"/>
-      <c r="F3" s="42"/>
-      <c r="G3" s="42"/>
-      <c r="H3" s="42"/>
-      <c r="I3" s="42"/>
-      <c r="J3" s="42"/>
-      <c r="K3" s="42"/>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A4" s="42" t="s">
+      <c r="B3" s="50"/>
+      <c r="C3" s="50"/>
+      <c r="D3" s="50"/>
+      <c r="E3" s="50"/>
+      <c r="F3" s="50"/>
+      <c r="G3" s="50"/>
+      <c r="H3" s="50"/>
+      <c r="I3" s="50"/>
+      <c r="J3" s="50"/>
+      <c r="K3" s="50"/>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" s="50" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="42"/>
-      <c r="C4" s="42"/>
-      <c r="D4" s="42"/>
-      <c r="E4" s="42"/>
-      <c r="F4" s="42"/>
-      <c r="G4" s="42"/>
-      <c r="H4" s="42"/>
-      <c r="I4" s="42"/>
-      <c r="J4" s="42"/>
-      <c r="K4" s="42"/>
-    </row>
-    <row r="5" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A5" s="43" t="s">
+      <c r="B4" s="50"/>
+      <c r="C4" s="50"/>
+      <c r="D4" s="50"/>
+      <c r="E4" s="50"/>
+      <c r="F4" s="50"/>
+      <c r="G4" s="50"/>
+      <c r="H4" s="50"/>
+      <c r="I4" s="50"/>
+      <c r="J4" s="50"/>
+      <c r="K4" s="50"/>
+    </row>
+    <row r="5" spans="1:16" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A5" s="51" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="43"/>
-      <c r="C5" s="43"/>
-      <c r="D5" s="43"/>
-      <c r="E5" s="43"/>
-      <c r="F5" s="43"/>
-      <c r="G5" s="43"/>
-      <c r="H5" s="43"/>
-      <c r="I5" s="43"/>
-      <c r="J5" s="43"/>
-      <c r="K5" s="43"/>
-    </row>
-    <row r="6" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A6" s="38" t="s">
+      <c r="B5" s="51"/>
+      <c r="C5" s="51"/>
+      <c r="D5" s="51"/>
+      <c r="E5" s="51"/>
+      <c r="F5" s="51"/>
+      <c r="G5" s="51"/>
+      <c r="H5" s="51"/>
+      <c r="I5" s="51"/>
+      <c r="J5" s="51"/>
+      <c r="K5" s="51"/>
+    </row>
+    <row r="6" spans="1:16" ht="18" x14ac:dyDescent="0.25">
+      <c r="A6" s="46" t="s">
         <v>59</v>
       </c>
-      <c r="B6" s="38"/>
-      <c r="C6" s="38"/>
-      <c r="D6" s="38"/>
-      <c r="E6" s="38"/>
-      <c r="F6" s="38"/>
+      <c r="B6" s="46"/>
+      <c r="C6" s="46"/>
+      <c r="D6" s="46"/>
+      <c r="E6" s="46"/>
+      <c r="F6" s="46"/>
       <c r="G6" s="10"/>
-      <c r="H6" s="39" t="s">
+      <c r="H6" s="47" t="s">
         <v>27</v>
       </c>
-      <c r="I6" s="39"/>
-      <c r="J6" s="39"/>
-      <c r="K6" s="39"/>
-    </row>
-    <row r="7" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="46" t="s">
+      <c r="I6" s="47"/>
+      <c r="J6" s="47"/>
+      <c r="K6" s="47"/>
+    </row>
+    <row r="7" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="41" t="s">
         <v>40</v>
       </c>
-      <c r="B7" s="46"/>
-      <c r="C7" s="46"/>
-      <c r="D7" s="46"/>
-      <c r="E7" s="46"/>
-      <c r="F7" s="46"/>
+      <c r="B7" s="41"/>
+      <c r="C7" s="41"/>
+      <c r="D7" s="41"/>
+      <c r="E7" s="41"/>
+      <c r="F7" s="41"/>
       <c r="G7" s="11"/>
-      <c r="H7" s="47" t="s">
+      <c r="H7" s="42" t="s">
         <v>58</v>
       </c>
-      <c r="I7" s="47"/>
-      <c r="J7" s="47"/>
-      <c r="K7" s="47"/>
-    </row>
-    <row r="8" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="I7" s="42"/>
+      <c r="J7" s="42"/>
+      <c r="K7" s="42"/>
+    </row>
+    <row r="8" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
         <v>5</v>
       </c>
@@ -1246,7 +1247,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="171.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" ht="173.25" x14ac:dyDescent="0.25">
       <c r="A9" s="16">
         <v>1</v>
       </c>
@@ -1263,7 +1264,7 @@
       <c r="J9" s="17"/>
       <c r="K9" s="17"/>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="16"/>
       <c r="B10" s="32" t="s">
         <v>36</v>
@@ -1304,7 +1305,7 @@
         <v>160.09797821843054</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="16"/>
       <c r="B11" s="32" t="s">
         <v>43</v>
@@ -1336,7 +1337,7 @@
       <c r="O11" s="36"/>
       <c r="P11" s="36"/>
     </row>
-    <row r="12" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="34" t="s">
         <v>16</v>
@@ -1361,7 +1362,7 @@
       </c>
       <c r="K12" s="5"/>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="16"/>
       <c r="B13" s="32" t="s">
         <v>42</v>
@@ -1379,7 +1380,7 @@
       </c>
       <c r="K13" s="17"/>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="16"/>
       <c r="B14" s="17"/>
       <c r="C14" s="17"/>
@@ -1392,7 +1393,7 @@
       <c r="J14" s="17"/>
       <c r="K14" s="17"/>
     </row>
-    <row r="15" spans="1:16" ht="109.2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:16" ht="110.25" x14ac:dyDescent="0.25">
       <c r="A15" s="16">
         <v>2</v>
       </c>
@@ -1409,7 +1410,7 @@
       <c r="J15" s="17"/>
       <c r="K15" s="17"/>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="16"/>
       <c r="B16" s="32" t="str">
         <f>B10</f>
@@ -1451,7 +1452,7 @@
         <v>160.09797821843054</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="16"/>
       <c r="B17" s="32" t="str">
         <f>B11</f>
@@ -1485,7 +1486,7 @@
       <c r="O17" s="36"/>
       <c r="P17" s="36"/>
     </row>
-    <row r="18" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
       <c r="B18" s="34" t="s">
         <v>16</v>
@@ -1510,7 +1511,7 @@
       </c>
       <c r="K18" s="5"/>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" s="16"/>
       <c r="B19" s="32" t="s">
         <v>22</v>
@@ -1528,7 +1529,7 @@
       </c>
       <c r="K19" s="17"/>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" s="16"/>
       <c r="B20" s="17"/>
       <c r="C20" s="17"/>
@@ -1541,7 +1542,7 @@
       <c r="J20" s="17"/>
       <c r="K20" s="17"/>
     </row>
-    <row r="21" spans="1:16" ht="93.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:16" ht="94.5" x14ac:dyDescent="0.25">
       <c r="A21" s="16">
         <v>3</v>
       </c>
@@ -1558,7 +1559,7 @@
       <c r="J21" s="17"/>
       <c r="K21" s="17"/>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="16"/>
       <c r="B22" s="32" t="str">
         <f>B16</f>
@@ -1600,7 +1601,7 @@
         <v>160.09797821843054</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" s="16"/>
       <c r="B23" s="32" t="str">
         <f>B17</f>
@@ -1634,7 +1635,7 @@
       <c r="O23" s="36"/>
       <c r="P23" s="36"/>
     </row>
-    <row r="24" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
       <c r="B24" s="34" t="s">
         <v>16</v>
@@ -1659,7 +1660,7 @@
       </c>
       <c r="K24" s="5"/>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" s="16"/>
       <c r="B25" s="32" t="s">
         <v>30</v>
@@ -1677,7 +1678,7 @@
       </c>
       <c r="K25" s="17"/>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" s="16"/>
       <c r="B26" s="32" t="s">
         <v>31</v>
@@ -1695,7 +1696,7 @@
       </c>
       <c r="K26" s="17"/>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" s="16"/>
       <c r="B27" s="32" t="s">
         <v>32</v>
@@ -1713,7 +1714,7 @@
       </c>
       <c r="K27" s="17"/>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" s="16"/>
       <c r="B28" s="32" t="s">
         <v>33</v>
@@ -1731,7 +1732,7 @@
       </c>
       <c r="K28" s="17"/>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A29" s="16"/>
       <c r="B29" s="32" t="s">
         <v>34</v>
@@ -1749,7 +1750,7 @@
       </c>
       <c r="K29" s="17"/>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" s="16"/>
       <c r="B30" s="17"/>
       <c r="C30" s="17"/>
@@ -1762,7 +1763,7 @@
       <c r="J30" s="17"/>
       <c r="K30" s="17"/>
     </row>
-    <row r="31" spans="1:16" ht="140.4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:16" ht="141.75" x14ac:dyDescent="0.25">
       <c r="A31" s="16">
         <v>4</v>
       </c>
@@ -1779,7 +1780,7 @@
       <c r="J31" s="17"/>
       <c r="K31" s="17"/>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" s="16"/>
       <c r="B32" s="32" t="str">
         <f>B22</f>
@@ -1819,7 +1820,7 @@
         <v>160.09797821843054</v>
       </c>
     </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33" s="16"/>
       <c r="B33" s="32" t="str">
         <f>B23</f>
@@ -1853,7 +1854,7 @@
       <c r="O33" s="36"/>
       <c r="P33" s="36"/>
     </row>
-    <row r="34" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2"/>
       <c r="B34" s="34" t="s">
         <v>16</v>
@@ -1878,7 +1879,7 @@
       </c>
       <c r="K34" s="5"/>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" s="16"/>
       <c r="B35" s="32" t="s">
         <v>30</v>
@@ -1896,7 +1897,7 @@
       </c>
       <c r="K35" s="17"/>
     </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" s="16"/>
       <c r="B36" s="32" t="s">
         <v>31</v>
@@ -1914,7 +1915,7 @@
       </c>
       <c r="K36" s="17"/>
     </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A37" s="16"/>
       <c r="B37" s="32" t="s">
         <v>38</v>
@@ -1932,7 +1933,7 @@
       </c>
       <c r="K37" s="17"/>
     </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A38" s="16"/>
       <c r="B38" s="32" t="s">
         <v>39</v>
@@ -1950,7 +1951,7 @@
       </c>
       <c r="K38" s="17"/>
     </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A39" s="16"/>
       <c r="B39" s="32" t="s">
         <v>33</v>
@@ -1968,7 +1969,7 @@
       </c>
       <c r="K39" s="17"/>
     </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" s="16"/>
       <c r="B40" s="17"/>
       <c r="C40" s="17"/>
@@ -1981,7 +1982,7 @@
       <c r="J40" s="17"/>
       <c r="K40" s="17"/>
     </row>
-    <row r="41" spans="1:16" ht="124.8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:16" ht="110.25" x14ac:dyDescent="0.25">
       <c r="A41" s="16">
         <v>5</v>
       </c>
@@ -1998,7 +1999,7 @@
       <c r="J41" s="17"/>
       <c r="K41" s="17"/>
     </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A42" s="16"/>
       <c r="B42" s="32" t="s">
         <v>56</v>
@@ -2024,7 +2025,7 @@
       <c r="O42" s="36"/>
       <c r="P42" s="36"/>
     </row>
-    <row r="43" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2"/>
       <c r="B43" s="34" t="s">
         <v>16</v>
@@ -2049,9 +2050,9 @@
       </c>
       <c r="K43" s="5"/>
     </row>
-    <row r="44" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A44" s="16"/>
-      <c r="B44" s="51" t="s">
+      <c r="B44" s="38" t="s">
         <v>57</v>
       </c>
       <c r="C44" s="17"/>
@@ -2067,7 +2068,7 @@
       </c>
       <c r="K44" s="17"/>
     </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A45" s="16"/>
       <c r="B45" s="32" t="s">
         <v>30</v>
@@ -2085,7 +2086,7 @@
       </c>
       <c r="K45" s="17"/>
     </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A46" s="16"/>
       <c r="B46" s="32" t="s">
         <v>31</v>
@@ -2103,7 +2104,7 @@
       </c>
       <c r="K46" s="17"/>
     </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A47" s="16"/>
       <c r="B47" s="17"/>
       <c r="C47" s="17"/>
@@ -2116,7 +2117,7 @@
       <c r="J47" s="17"/>
       <c r="K47" s="17"/>
     </row>
-    <row r="48" spans="1:16" ht="124.8" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:16" ht="110.25" x14ac:dyDescent="0.25">
       <c r="A48" s="16">
         <v>6</v>
       </c>
@@ -2133,7 +2134,7 @@
       <c r="J48" s="17"/>
       <c r="K48" s="17"/>
     </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A49" s="16"/>
       <c r="B49" s="32" t="s">
         <v>52</v>
@@ -2159,7 +2160,7 @@
       <c r="O49" s="36"/>
       <c r="P49" s="36"/>
     </row>
-    <row r="50" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2"/>
       <c r="B50" s="34" t="s">
         <v>16</v>
@@ -2184,9 +2185,9 @@
       </c>
       <c r="K50" s="5"/>
     </row>
-    <row r="51" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A51" s="16"/>
-      <c r="B51" s="51" t="s">
+      <c r="B51" s="38" t="s">
         <v>54</v>
       </c>
       <c r="C51" s="17"/>
@@ -2202,7 +2203,7 @@
       </c>
       <c r="K51" s="17"/>
     </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A52" s="16"/>
       <c r="B52" s="32" t="s">
         <v>30</v>
@@ -2220,7 +2221,7 @@
       </c>
       <c r="K52" s="17"/>
     </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A53" s="16"/>
       <c r="B53" s="32" t="s">
         <v>31</v>
@@ -2238,7 +2239,7 @@
       </c>
       <c r="K53" s="17"/>
     </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A54" s="16"/>
       <c r="B54" s="17"/>
       <c r="C54" s="17"/>
@@ -2251,7 +2252,7 @@
       <c r="J54" s="17"/>
       <c r="K54" s="17"/>
     </row>
-    <row r="55" spans="1:16" ht="121.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:16" ht="121.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="16">
         <v>7</v>
       </c>
@@ -2268,7 +2269,7 @@
       <c r="J55" s="17"/>
       <c r="K55" s="17"/>
     </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A56" s="16"/>
       <c r="B56" s="32" t="s">
         <v>45</v>
@@ -2300,7 +2301,7 @@
       <c r="O56" s="36"/>
       <c r="P56" s="36"/>
     </row>
-    <row r="57" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2"/>
       <c r="B57" s="34" t="s">
         <v>16</v>
@@ -2325,9 +2326,9 @@
       </c>
       <c r="K57" s="5"/>
     </row>
-    <row r="58" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A58" s="16"/>
-      <c r="B58" s="51" t="s">
+      <c r="B58" s="38" t="s">
         <v>47</v>
       </c>
       <c r="C58" s="17"/>
@@ -2343,7 +2344,7 @@
       </c>
       <c r="K58" s="17"/>
     </row>
-    <row r="59" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A59" s="16"/>
       <c r="B59" s="32" t="s">
         <v>34</v>
@@ -2361,7 +2362,7 @@
       </c>
       <c r="K59" s="17"/>
     </row>
-    <row r="60" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A60" s="16"/>
       <c r="B60" s="32" t="s">
         <v>48</v>
@@ -2379,7 +2380,7 @@
       </c>
       <c r="K60" s="17"/>
     </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A61" s="16"/>
       <c r="B61" s="32" t="s">
         <v>49</v>
@@ -2397,7 +2398,7 @@
       </c>
       <c r="K61" s="17"/>
     </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A62" s="16"/>
       <c r="B62" s="32" t="s">
         <v>50</v>
@@ -2415,7 +2416,7 @@
       </c>
       <c r="K62" s="17"/>
     </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A63" s="16"/>
       <c r="B63" s="17"/>
       <c r="C63" s="17"/>
@@ -2428,7 +2429,7 @@
       <c r="J63" s="17"/>
       <c r="K63" s="17"/>
     </row>
-    <row r="64" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="2">
         <v>8</v>
       </c>
@@ -2457,7 +2458,7 @@
       </c>
       <c r="K64" s="5"/>
     </row>
-    <row r="65" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A65" s="2"/>
       <c r="B65" s="8"/>
       <c r="C65" s="3"/>
@@ -2470,7 +2471,7 @@
       <c r="J65" s="18"/>
       <c r="K65" s="5"/>
     </row>
-    <row r="66" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2">
         <v>9</v>
       </c>
@@ -2499,7 +2500,7 @@
       </c>
       <c r="K66" s="5"/>
     </row>
-    <row r="67" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A67" s="2"/>
       <c r="B67" s="8"/>
       <c r="C67" s="3"/>
@@ -2512,7 +2513,7 @@
       <c r="J67" s="18"/>
       <c r="K67" s="5"/>
     </row>
-    <row r="68" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A68" s="21"/>
       <c r="B68" s="22" t="s">
         <v>21</v>
@@ -2530,7 +2531,7 @@
       </c>
       <c r="K68" s="25"/>
     </row>
-    <row r="69" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:19" x14ac:dyDescent="0.25">
       <c r="M69" s="20"/>
       <c r="N69" s="20"/>
       <c r="O69" s="20"/>
@@ -2539,16 +2540,16 @@
       <c r="R69" s="20"/>
       <c r="S69" s="20"/>
     </row>
-    <row r="70" spans="1:19" s="20" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:19" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="26"/>
       <c r="B70" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="C70" s="44">
+      <c r="C70" s="39">
         <f>J68</f>
         <v>483034.47031716217</v>
       </c>
-      <c r="D70" s="45"/>
+      <c r="D70" s="40"/>
       <c r="E70" s="9">
         <v>100</v>
       </c>
@@ -2566,72 +2567,79 @@
       <c r="R70" s="19"/>
       <c r="S70" s="19"/>
     </row>
-    <row r="71" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B71" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="C71" s="48">
-        <v>300000</v>
-      </c>
-      <c r="D71" s="49"/>
+      <c r="C71" s="43">
+        <v>425000</v>
+      </c>
+      <c r="D71" s="44"/>
       <c r="E71" s="9"/>
     </row>
-    <row r="72" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B72" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="C72" s="48">
+      <c r="C72" s="43">
         <f>C71-C74-C75</f>
-        <v>285000</v>
-      </c>
-      <c r="D72" s="49"/>
+        <v>403750</v>
+      </c>
+      <c r="D72" s="44"/>
       <c r="E72" s="9">
         <f>C72/C70*100</f>
-        <v>59.002000377502661</v>
-      </c>
-    </row>
-    <row r="73" spans="1:19" x14ac:dyDescent="0.3">
+        <v>83.586167201462104</v>
+      </c>
+    </row>
+    <row r="73" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B73" s="27" t="s">
         <v>35</v>
       </c>
-      <c r="C73" s="50">
+      <c r="C73" s="45">
         <f>C70-C72</f>
-        <v>198034.47031716217</v>
-      </c>
-      <c r="D73" s="50"/>
+        <v>79284.470317162166</v>
+      </c>
+      <c r="D73" s="45"/>
       <c r="E73" s="9">
         <f>100-E72</f>
-        <v>40.997999622497339</v>
-      </c>
-    </row>
-    <row r="74" spans="1:19" x14ac:dyDescent="0.3">
+        <v>16.413832798537896</v>
+      </c>
+    </row>
+    <row r="74" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B74" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="C74" s="44">
+      <c r="C74" s="39">
         <f>C71*0.03</f>
-        <v>9000</v>
-      </c>
-      <c r="D74" s="45"/>
+        <v>12750</v>
+      </c>
+      <c r="D74" s="40"/>
       <c r="E74" s="9">
         <v>3</v>
       </c>
     </row>
-    <row r="75" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B75" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="C75" s="44">
+      <c r="C75" s="39">
         <f>C71*0.02</f>
-        <v>6000</v>
-      </c>
-      <c r="D75" s="45"/>
+        <v>8500</v>
+      </c>
+      <c r="D75" s="40"/>
       <c r="E75" s="9">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
     <mergeCell ref="C74:D74"/>
     <mergeCell ref="C75:D75"/>
     <mergeCell ref="A7:F7"/>
@@ -2640,13 +2648,6 @@
     <mergeCell ref="C71:D71"/>
     <mergeCell ref="C72:D72"/>
     <mergeCell ref="C73:D73"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="H6:K6"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
   </mergeCells>
   <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
   <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>

</xml_diff>